<commit_message>
Committing & purshing for backup purposes
</commit_message>
<xml_diff>
--- a/Time_Tracking/WorkHours_Calculator_2026.xlsx
+++ b/Time_Tracking/WorkHours_Calculator_2026.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Git_Repositories\PubDev\Time_Tracking\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B7696F93-5776-434A-A5EC-38930E2832A0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{73A61724-6549-4F88-8E4B-22B34DE23C07}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="3840" yWindow="1575" windowWidth="24360" windowHeight="16905" xr2:uid="{F0FEE646-CA9E-4872-A8E1-626BBC6FFE10}"/>
   </bookViews>
@@ -67,7 +67,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="128" uniqueCount="22">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="128" uniqueCount="25">
   <si>
     <t>In</t>
   </si>
@@ -212,6 +212,31 @@
   </si>
   <si>
     <t>Hours &gt; 40</t>
+  </si>
+  <si>
+    <t>Pre-Lunch
+Hours</t>
+  </si>
+  <si>
+    <t>Post-Lunch
+Hours</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Time Off
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>(PTO, Holiday, Bereavement, etc.)</t>
+    </r>
   </si>
 </sst>
 </file>
@@ -1654,15 +1679,17 @@
   <dimension ref="A1:M25"/>
   <sheetFormatPr defaultRowHeight="23.25" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="18.42578125" style="18" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="17.42578125" style="18" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="13.140625" style="20" bestFit="1" customWidth="1"/>
-    <col min="3" max="5" width="15" style="20" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="15" style="20" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="14.5703125" style="20" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.7109375" style="20" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="18.42578125" style="20" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="30.5703125" style="20" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="13.7109375" style="20" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="35.7109375" style="20" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="15.7109375" style="20" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="20.140625" style="20" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="17.7109375" style="20" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="11" customWidth="1"/>
+    <col min="11" max="11" width="11" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="20.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -1687,13 +1714,13 @@
         <v>16</v>
       </c>
       <c r="G1" s="6" t="s">
-        <v>15</v>
+        <v>24</v>
       </c>
       <c r="H1" s="6" t="s">
-        <v>12</v>
-      </c>
-      <c r="I1" s="3" t="s">
-        <v>13</v>
+        <v>22</v>
+      </c>
+      <c r="I1" s="6" t="s">
+        <v>23</v>
       </c>
       <c r="J1" s="3" t="s">
         <v>14</v>
@@ -1757,35 +1784,39 @@
       <c r="B3" s="8">
         <v>0.28819444444444442</v>
       </c>
-      <c r="C3" s="8"/>
-      <c r="D3" s="8"/>
+      <c r="C3" s="8">
+        <v>0.52083333333333337</v>
+      </c>
+      <c r="D3" s="8">
+        <v>0.55208333333333337</v>
+      </c>
       <c r="E3" s="9">
         <v>0.66666666666666663</v>
       </c>
       <c r="F3" s="30">
         <f t="shared" ref="F3:F6" si="0">IF(G3 &gt;= 8, 4 + COUNT(B3:E3), IF(AND(G3 &gt;= 4, G3 &lt;= 7), 2 + COUNT(B3:E3), COUNT(B3:E3)))</f>
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G3" s="10"/>
       <c r="H3" s="10">
         <f>SUM(C3 - B3) * 24</f>
-        <v>-6.9166666666666661</v>
+        <v>5.5833333333333348</v>
       </c>
       <c r="I3" s="11">
         <f>SUM(E3 - D3) * 24</f>
-        <v>16</v>
+        <v>2.7499999999999982</v>
       </c>
       <c r="J3" s="12">
         <f t="shared" ref="J3:J6" si="1">H3 + I3 + G3</f>
-        <v>9.0833333333333339</v>
-      </c>
-      <c r="K3" s="13" t="str">
+        <v>8.3333333333333321</v>
+      </c>
+      <c r="K3" s="13">
         <f>IF(AND(C3 &lt;&gt; "", D3 &lt;&gt; ""), (SUM(D3 - C3) * 1440), " - ")</f>
-        <v xml:space="preserve"> - </v>
-      </c>
-      <c r="L3" s="14" t="str">
+        <v>45</v>
+      </c>
+      <c r="L3" s="14">
         <f>IF(AND((B3 &lt;&gt; ""), (C3 &lt;&gt; ""), (D3 &lt;&gt; ""), (E3 &lt;&gt; "")), IF((((8 - J3) * 60) + 1) &gt; 0, (((8 - J3) * 60) + 1), (((8 - J3) * 60) - 1)), "-")</f>
-        <v>-</v>
+        <v>-20.999999999999929</v>
       </c>
     </row>
     <row r="4" spans="1:13" x14ac:dyDescent="0.35">
@@ -1906,7 +1937,7 @@
       </c>
       <c r="J7" s="22">
         <f>SUM(J2:J6)</f>
-        <v>26.38333333333334</v>
+        <v>25.633333333333333</v>
       </c>
     </row>
     <row r="8" spans="1:13" ht="24" thickBot="1" x14ac:dyDescent="0.4"/>
@@ -1918,7 +1949,7 @@
       </c>
       <c r="J9" s="25">
         <f>40-J7</f>
-        <v>13.61666666666666</v>
+        <v>14.366666666666667</v>
       </c>
       <c r="K9" s="26"/>
     </row>

</xml_diff>

<commit_message>
Comitting & pushing for backup purposes
</commit_message>
<xml_diff>
--- a/Time_Tracking/WorkHours_Calculator_2026.xlsx
+++ b/Time_Tracking/WorkHours_Calculator_2026.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Git_Repositories\PubDev\Time_Tracking\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0CFC1A54-34DB-4091-BA74-75525E4CB85B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7518B91C-73EB-4E96-B4F7-5A1327CB3BEA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="41595" yWindow="1845" windowWidth="24360" windowHeight="16905" xr2:uid="{F0FEE646-CA9E-4872-A8E1-626BBC6FFE10}"/>
+    <workbookView xWindow="4860" yWindow="1575" windowWidth="24360" windowHeight="16905" xr2:uid="{F0FEE646-CA9E-4872-A8E1-626BBC6FFE10}"/>
   </bookViews>
   <sheets>
     <sheet name="20260309" sheetId="10" r:id="rId1"/>
@@ -1915,35 +1915,39 @@
       <c r="B6" s="8">
         <v>0.28819444444444442</v>
       </c>
-      <c r="C6" s="8"/>
-      <c r="D6" s="8"/>
+      <c r="C6" s="8">
+        <v>0.50208333333333333</v>
+      </c>
+      <c r="D6" s="8">
+        <v>0.53263888888888888</v>
+      </c>
       <c r="E6" s="9">
         <v>0.66666666666666663</v>
       </c>
       <c r="F6" s="30">
         <f t="shared" si="0"/>
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G6" s="10"/>
       <c r="H6" s="10">
         <f>SUM(C6 - B6) * 24</f>
-        <v>-6.9166666666666661</v>
+        <v>5.1333333333333337</v>
       </c>
       <c r="I6" s="11">
         <f t="shared" si="3"/>
-        <v>16</v>
+        <v>3.2166666666666659</v>
       </c>
       <c r="J6" s="12">
         <f t="shared" si="1"/>
-        <v>9.0833333333333339</v>
-      </c>
-      <c r="K6" s="13" t="str">
+        <v>8.35</v>
+      </c>
+      <c r="K6" s="13">
         <f t="shared" si="4"/>
-        <v xml:space="preserve"> - </v>
-      </c>
-      <c r="L6" s="14" t="str">
+        <v>44</v>
+      </c>
+      <c r="L6" s="14">
         <f>IF(AND((B6 &lt;&gt; ""), (C6 &lt;&gt; ""), (D6 &lt;&gt; ""), (E6 &lt;&gt; "")), IF((((8 - J6) * 60) + 1) &gt; 0, (((8 - J6) * 60) + 1), (((8 - J6) * 60) - 1)), "-")</f>
-        <v>-</v>
+        <v>-21.999999999999979</v>
       </c>
     </row>
     <row r="7" spans="1:13" ht="36.75" thickBot="1" x14ac:dyDescent="0.6">
@@ -1953,7 +1957,7 @@
       </c>
       <c r="J7" s="22">
         <f>SUM(J2:J6)</f>
-        <v>42.31666666666667</v>
+        <v>41.583333333333336</v>
       </c>
     </row>
     <row r="8" spans="1:13" ht="24" thickBot="1" x14ac:dyDescent="0.4"/>
@@ -1965,7 +1969,7 @@
       </c>
       <c r="J9" s="25">
         <f>40-J7</f>
-        <v>-2.31666666666667</v>
+        <v>-1.5833333333333357</v>
       </c>
       <c r="K9" s="26"/>
     </row>
@@ -1975,7 +1979,7 @@
       </c>
       <c r="J10" s="25">
         <f>IF(J7 &lt; 40, "-", J7-40)</f>
-        <v>2.31666666666667</v>
+        <v>1.5833333333333357</v>
       </c>
     </row>
     <row r="15" spans="1:13" x14ac:dyDescent="0.35">

</xml_diff>

<commit_message>
Committing & pushing fo rbackup purposes
</commit_message>
<xml_diff>
--- a/Time_Tracking/WorkHours_Calculator_2026.xlsx
+++ b/Time_Tracking/WorkHours_Calculator_2026.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Git_Repositories\PubDev\Time_Tracking\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E3B54FF9-C5DE-4D3E-8973-0457ADA34CF1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A944511F-090B-4506-9335-BEB061EDD74A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="3615" yWindow="2010" windowWidth="27180" windowHeight="16905" xr2:uid="{F0FEE646-CA9E-4872-A8E1-626BBC6FFE10}"/>
   </bookViews>
@@ -2194,34 +2194,42 @@
         <f ca="1">_xlfn.CONCAT(TEXT(A1 + 1, "ddd"), " (", DAY(A1 + 1), IF(OR(AND(DAY(A1 + 1) &gt; 23, DAY(A1 + 1) &lt; 31), AND(DAY(A1 + 1) &gt; 3, DAY(A1 + 1) &lt; 21)), "th", LOOKUP(DAY(A1 + 1), {1,"st";2,"nd";3,"rd";21,"st";22,"nd";23,"rd";31,"st"})), ")")</f>
         <v>Thu (9th)</v>
       </c>
-      <c r="B3" s="8"/>
-      <c r="C3" s="8"/>
-      <c r="D3" s="8"/>
-      <c r="E3" s="9"/>
+      <c r="B3" s="8">
+        <v>0.28819444444444442</v>
+      </c>
+      <c r="C3" s="8">
+        <v>0.49444444444444446</v>
+      </c>
+      <c r="D3" s="8">
+        <v>0.52500000000000002</v>
+      </c>
+      <c r="E3" s="9">
+        <v>0.66666666666666663</v>
+      </c>
       <c r="F3" s="30">
         <f t="shared" ref="F3:F6" si="0">IF(G3 &gt;= 8, 4 + COUNT(B3:E3), IF(AND(G3 &gt;= 4, G3 &lt;= 7), 2 + COUNT(B3:E3), COUNT(B3:E3)))</f>
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="G3" s="10"/>
       <c r="H3" s="10">
         <f>SUM(C3 - B3) * 24</f>
-        <v>0</v>
+        <v>4.9500000000000011</v>
       </c>
       <c r="I3" s="11">
         <f>SUM(E3 - D3) * 24</f>
-        <v>0</v>
+        <v>3.3999999999999986</v>
       </c>
       <c r="J3" s="12">
         <f t="shared" ref="J3:J6" si="1">H3 + I3 + G3</f>
-        <v>0</v>
-      </c>
-      <c r="K3" s="13" t="str">
+        <v>8.35</v>
+      </c>
+      <c r="K3" s="13">
         <f>IF(AND(C3 &lt;&gt; "", D3 &lt;&gt; ""), (SUM(D3 - C3) * 1440), " - ")</f>
-        <v xml:space="preserve"> - </v>
-      </c>
-      <c r="L3" s="14" t="str">
+        <v>44</v>
+      </c>
+      <c r="L3" s="14">
         <f>IF(AND((B3 &lt;&gt; ""), (C3 &lt;&gt; ""), (D3 &lt;&gt; ""), (E3 &lt;&gt; "")), IF((((8 - J3) * 60) + 1) &gt; 0, (((8 - J3) * 60) + 1), (((8 - J3) * 60) - 1)), "-")</f>
-        <v>-</v>
+        <v>-21.999999999999979</v>
       </c>
     </row>
     <row r="4" spans="1:13" x14ac:dyDescent="0.35">
@@ -2336,11 +2344,11 @@
       </c>
       <c r="J7" s="22">
         <f>SUM(J2:J6)</f>
-        <v>8.3333333333333321</v>
+        <v>16.68333333333333</v>
       </c>
       <c r="K7" s="25">
         <f>IF(SUM(K2:K6) &lt;&gt; 0, ((60*5) - SUM(K2:K6)) / 60, 0)</f>
-        <v>4.25</v>
+        <v>3.5166666666666666</v>
       </c>
     </row>
     <row r="8" spans="1:13" ht="24" thickBot="1" x14ac:dyDescent="0.4"/>
@@ -2352,7 +2360,7 @@
       </c>
       <c r="J9" s="25">
         <f>40-J7</f>
-        <v>31.666666666666668</v>
+        <v>23.31666666666667</v>
       </c>
       <c r="K9" s="26"/>
     </row>

</xml_diff>